<commit_message>
Daily NSE scan: 2026-10-09
</commit_message>
<xml_diff>
--- a/output/2026-10-09/enriched_analysis.xlsx
+++ b/output/2026-10-09/enriched_analysis.xlsx
@@ -929,10 +929,10 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>2.234</v>
+        <v>2.233</v>
       </c>
       <c r="W2" t="n">
-        <v>2820</v>
+        <v>2821</v>
       </c>
       <c r="X2" t="n">
         <v>22.1</v>
@@ -1396,10 +1396,10 @@
         <v>0.046</v>
       </c>
       <c r="W4" t="n">
-        <v>2903</v>
+        <v>2902</v>
       </c>
       <c r="X4" t="n">
-        <v>9.98</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="Y4" t="n">
         <v>36</v>
@@ -2087,13 +2087,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>0.137</v>
+        <v>0.136</v>
       </c>
       <c r="W7" t="n">
-        <v>2297</v>
+        <v>2300</v>
       </c>
       <c r="X7" t="n">
-        <v>20.1</v>
+        <v>20.2</v>
       </c>
       <c r="Y7" t="n">
         <v>-3</v>
@@ -2319,13 +2319,13 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>1.167</v>
+        <v>1.173</v>
       </c>
       <c r="W8" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="X8" t="n">
-        <v>7.3</v>
+        <v>7.28</v>
       </c>
       <c r="Y8" t="n">
         <v>17</v>
@@ -2551,13 +2551,13 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>1.18</v>
+        <v>1.188</v>
       </c>
       <c r="W9" t="n">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="X9" t="n">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="Y9" t="n">
         <v>22</v>
@@ -2786,7 +2786,7 @@
         <v>0.048</v>
       </c>
       <c r="W10" t="n">
-        <v>14958</v>
+        <v>14952</v>
       </c>
       <c r="X10" t="n">
         <v>38.1</v>
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>2.338</v>
+        <v>2.348</v>
       </c>
       <c r="W11" t="n">
-        <v>2511</v>
+        <v>2500</v>
       </c>
       <c r="X11" t="n">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Y11" t="n">
         <v>6</v>
@@ -3250,10 +3250,10 @@
         <v>0.067</v>
       </c>
       <c r="W12" t="n">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="X12" t="n">
-        <v>21.4</v>
+        <v>21.3</v>
       </c>
       <c r="Y12" t="n">
         <v>19</v>
@@ -3477,13 +3477,13 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>0.052</v>
+        <v>0.051</v>
       </c>
       <c r="W13" t="n">
-        <v>1594</v>
+        <v>1602</v>
       </c>
       <c r="X13" t="n">
-        <v>21.5</v>
+        <v>21.6</v>
       </c>
       <c r="Y13" t="n">
         <v>55</v>
@@ -3709,10 +3709,10 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="W14" t="n">
-        <v>2564</v>
+        <v>2561</v>
       </c>
       <c r="X14" t="n">
         <v>21</v>
@@ -3944,7 +3944,7 @@
         <v>0.06900000000000001</v>
       </c>
       <c r="W15" t="n">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="X15" t="n">
         <v>36.7</v>
@@ -4173,10 +4173,10 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>2.946</v>
+        <v>2.95</v>
       </c>
       <c r="W16" t="n">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="X16" t="n">
         <v>20.2</v>
@@ -4399,13 +4399,13 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>0.193</v>
+        <v>0.188</v>
       </c>
       <c r="W17" t="n">
-        <v>574</v>
+        <v>590</v>
       </c>
       <c r="X17" t="n">
-        <v>48</v>
+        <v>49.3</v>
       </c>
       <c r="Y17" t="n">
         <v>3</v>
@@ -4631,13 +4631,13 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0.092</v>
+        <v>0.091</v>
       </c>
       <c r="W18" t="n">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="X18" t="n">
-        <v>10.1</v>
+        <v>10.2</v>
       </c>
       <c r="Y18" t="n">
         <v>-5</v>
@@ -4866,7 +4866,7 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W19" t="n">
-        <v>54545</v>
+        <v>54563</v>
       </c>
       <c r="X19" t="n">
         <v>46.2</v>
@@ -5095,10 +5095,10 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.671</v>
+        <v>0.673</v>
       </c>
       <c r="W20" t="n">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="X20" t="n">
         <v>10.8</v>
@@ -5330,10 +5330,10 @@
         <v>0.093</v>
       </c>
       <c r="W21" t="n">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="X21" t="n">
-        <v>40.1</v>
+        <v>40.2</v>
       </c>
       <c r="Y21" t="n">
         <v>17</v>
@@ -5553,13 +5553,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>1.033</v>
+        <v>1.044</v>
       </c>
       <c r="W22" t="n">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="X22" t="n">
-        <v>5.63</v>
+        <v>5.56</v>
       </c>
       <c r="Y22" t="n">
         <v>31</v>
@@ -5781,13 +5781,13 @@
         </is>
       </c>
       <c r="V23" t="n">
-        <v>0.309</v>
+        <v>0.325</v>
       </c>
       <c r="W23" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="X23" t="n">
-        <v>24.9</v>
+        <v>23.6</v>
       </c>
       <c r="Y23" t="n">
         <v>12</v>
@@ -6013,13 +6013,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.376</v>
+        <v>0.375</v>
       </c>
       <c r="W24" t="n">
-        <v>1045</v>
+        <v>1048</v>
       </c>
       <c r="X24" t="n">
-        <v>53.2</v>
+        <v>53.4</v>
       </c>
       <c r="Y24" t="n">
         <v>21</v>
@@ -6245,13 +6245,13 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.524</v>
+        <v>0.52</v>
       </c>
       <c r="W25" t="n">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="X25" t="n">
-        <v>35.4</v>
+        <v>35.6</v>
       </c>
       <c r="Y25" t="n">
         <v>21</v>
@@ -6477,13 +6477,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.529</v>
+        <v>0.534</v>
       </c>
       <c r="W26" t="n">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="X26" t="n">
-        <v>35.2</v>
+        <v>34.8</v>
       </c>
       <c r="Y26" t="n">
         <v>-44</v>
@@ -6709,10 +6709,10 @@
         </is>
       </c>
       <c r="V27" t="n">
-        <v>0.132</v>
+        <v>0.131</v>
       </c>
       <c r="W27" t="n">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="X27" t="n">
         <v>13.4</v>
@@ -6944,7 +6944,7 @@
         <v>0.042</v>
       </c>
       <c r="W28" t="n">
-        <v>1640</v>
+        <v>1637</v>
       </c>
       <c r="X28" t="n">
         <v>21.4</v>
@@ -7173,13 +7173,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.275</v>
+        <v>0.274</v>
       </c>
       <c r="W29" t="n">
-        <v>948</v>
+        <v>951</v>
       </c>
       <c r="X29" t="n">
-        <v>25.8</v>
+        <v>25.9</v>
       </c>
       <c r="Y29" t="n">
         <v>9</v>
@@ -7405,10 +7405,10 @@
         </is>
       </c>
       <c r="V30" t="n">
-        <v>1.86</v>
+        <v>1.893</v>
       </c>
       <c r="W30" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="n">
@@ -7861,13 +7861,13 @@
         </is>
       </c>
       <c r="V32" t="n">
-        <v>0.656</v>
+        <v>0.669</v>
       </c>
       <c r="W32" t="n">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="X32" t="n">
-        <v>1156</v>
+        <v>1131</v>
       </c>
       <c r="Y32" t="n">
         <v>-61</v>
@@ -8089,13 +8089,13 @@
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0.245</v>
+        <v>0.246</v>
       </c>
       <c r="W33" t="n">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="X33" t="n">
-        <v>14</v>
+        <v>13.9</v>
       </c>
       <c r="Y33" t="n">
         <v>16</v>
@@ -8324,7 +8324,7 @@
         <v>0.234</v>
       </c>
       <c r="W34" t="n">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="X34" t="n">
         <v>18.1</v>
@@ -8556,7 +8556,7 @@
         <v>0.042</v>
       </c>
       <c r="W35" t="n">
-        <v>3178</v>
+        <v>3176</v>
       </c>
       <c r="X35" t="n">
         <v>18.8</v>
@@ -8785,13 +8785,13 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>0.376</v>
+        <v>0.374</v>
       </c>
       <c r="W36" t="n">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="X36" t="n">
-        <v>92.09999999999999</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="Y36" t="n">
         <v>246</v>
@@ -9020,10 +9020,10 @@
         <v>0.869</v>
       </c>
       <c r="W37" t="n">
-        <v>3638</v>
+        <v>3636</v>
       </c>
       <c r="X37" t="n">
-        <v>25.5</v>
+        <v>25.4</v>
       </c>
       <c r="Y37" t="n">
         <v>2</v>
@@ -9252,7 +9252,7 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>5237</v>
+        <v>5239</v>
       </c>
       <c r="X38" t="n">
         <v>12.3</v>
@@ -9484,7 +9484,7 @@
         <v>0.011</v>
       </c>
       <c r="W39" t="n">
-        <v>4078</v>
+        <v>4068</v>
       </c>
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="n">
@@ -9711,13 +9711,13 @@
         </is>
       </c>
       <c r="V40" t="n">
-        <v>0.109</v>
+        <v>0.11</v>
       </c>
       <c r="W40" t="n">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="X40" t="n">
-        <v>7.34</v>
+        <v>7.28</v>
       </c>
       <c r="Y40" t="n">
         <v>118</v>
@@ -10171,13 +10171,13 @@
         </is>
       </c>
       <c r="V42" t="n">
-        <v>0.08</v>
+        <v>0.079</v>
       </c>
       <c r="W42" t="n">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="X42" t="n">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
       <c r="Y42" t="n">
         <v>-8</v>
@@ -10403,10 +10403,10 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.104</v>
+        <v>0.105</v>
       </c>
       <c r="W43" t="n">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="X43" t="n">
         <v>26.2</v>
@@ -10635,10 +10635,10 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.053</v>
+        <v>0.052</v>
       </c>
       <c r="W44" t="n">
-        <v>932</v>
+        <v>942</v>
       </c>
       <c r="X44" t="inlineStr"/>
       <c r="Y44" t="n">
@@ -10868,7 +10868,7 @@
         <v>0</v>
       </c>
       <c r="W45" t="n">
-        <v>3737</v>
+        <v>3735</v>
       </c>
       <c r="X45" t="n">
         <v>84.09999999999999</v>
@@ -11100,7 +11100,7 @@
         <v>0.006</v>
       </c>
       <c r="W46" t="n">
-        <v>4776</v>
+        <v>4771</v>
       </c>
       <c r="X46" t="n">
         <v>12.3</v>
@@ -11328,7 +11328,7 @@
         <v>0</v>
       </c>
       <c r="W47" t="n">
-        <v>103165</v>
+        <v>103029</v>
       </c>
       <c r="X47" t="n">
         <v>29.7</v>
@@ -11557,10 +11557,10 @@
         </is>
       </c>
       <c r="V48" t="n">
-        <v>0.227</v>
+        <v>0.225</v>
       </c>
       <c r="W48" t="n">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="X48" t="n">
         <v>23.6</v>

</xml_diff>